<commit_message>
Actualiza comparativo de identificación de normas VF
</commit_message>
<xml_diff>
--- a/LexIA_Diario/Comparativo de identificación de normas VF (1).xlsx
+++ b/LexIA_Diario/Comparativo de identificación de normas VF (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://interbankpe-my.sharepoint.com/personal/shernandez2_intercorp_com_pe/Documents/PLAFT/GenIA/Normativo/LexIA_Diario/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://interbankpe-my.sharepoint.com/personal/shernandez2_intercorp_com_pe/Documents/PLAFT/Interbank/LexIA_Diario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="531" documentId="11_FF9E2F5B496FDA3AB52BB0B2B6FDBBEC0357B1A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E48F9C1E-50FD-44CB-BF18-B32E140B0745}"/>
+  <xr:revisionPtr revIDLastSave="594" documentId="11_FF9E2F5B496FDA3AB52BB0B2B6FDBBEC0357B1A8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9A8DE30-9B39-424F-931B-22FD144B61E9}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1095" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Hoja1!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Hoja2!$B$3:$H$13</definedName>
   </definedNames>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2624" uniqueCount="1027">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2662" uniqueCount="1046">
   <si>
     <t>Dia</t>
   </si>
@@ -3091,6 +3091,69 @@
   <si>
     <t>Índice de reajuste diario a que se refiere el artículo 240° de la Ley General del Sistema Financiero y del Sistema de Seguros, correspondiente al mes de setiembre de
 2026</t>
+  </si>
+  <si>
+    <t>Circular SBS</t>
+  </si>
+  <si>
+    <t>Nº F-618-2026</t>
+  </si>
+  <si>
+    <t>Actualización del monto máximo de cobertura del Fondo de Seguro de Depósitos correspondiente al trimestre setiembre 2026 - noviembre 2026</t>
+  </si>
+  <si>
+    <t>SBS 02117-2026</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Autorizan la difusión en consulta pública del proyecto de norma PLAFT aplicable a laboratorios y empresas vinculadas a insumos químicos y bienes fiscalizados.</t>
+  </si>
+  <si>
+    <t>Nº 125-2026-PCM</t>
+  </si>
+  <si>
+    <t>Decreto Supremo que declara el Estado de Emergencia en los distritos de Pangoa
+y Río Tambo de la provincia de Satipo del departamento de Junín; en los distritos
+de Megantoni, Kumpirushiato, Echarate, Villa Virgen, Villa Kintiarina, Manitea,
+Kimbiri y Cielo Punco de la provincia de La Convención del departamento de Cusco;
+y en los distritos de Ayna, Santa Rosa, Anchihuay, Río Magdalena, Samugari, Anco
+y Unión Progreso de la provincia de La Mar del departamento de Ayacucho</t>
+  </si>
+  <si>
+    <t>Nº 126-2026-PCM</t>
+  </si>
+  <si>
+    <t>Decreto Supremo que declara el Estado de Emergencia en los distritos de Piura,Castilla, Veintiséis de Octubre y Catacaos de la provincia de Piura, en los distritos
+de Sullana y Bellavista de la provincia de Sullana, y en las provincias de Paita y Talara del departamento de Piura y dicta otras disposiciones</t>
+  </si>
+  <si>
+    <t>N° 003-2026-EF/30</t>
+  </si>
+  <si>
+    <t>Aprueban el Set Completo de las Normas Internacionales de Información Financiera versión 2026, que incluye el Marco Conceptual para la Información Financiera</t>
+  </si>
+  <si>
+    <t>Resolución Ministerial</t>
+  </si>
+  <si>
+    <t>Nº 808-2026/MINSA</t>
+  </si>
+  <si>
+    <t>Aprueban Relación de Servicios que pueden ejecutarse mediante el mecanismo de Obras por Impuestos, en el marco de lo dispuesto en el numeral 4.2 del artículo 4 y la Quinta Disposición Complementaria Final del Decreto de Urgencia N° 010-2026</t>
+  </si>
+  <si>
+    <t>N° 544-2026-MINEDU</t>
+  </si>
+  <si>
+    <t>Aprueban la “Relación de Servicios que pueden ejecutarse mediante el mecanismo de Obras por Impuestos en el marco del Decreto de Urgencia N° 010-2026 para atender el Fenómeno El Niño” y su contenido mínimo</t>
+  </si>
+  <si>
+    <t>N° 000332-2026-MC</t>
+  </si>
+  <si>
+    <t>Aprueban listado de servicios que pueden ejecutarse mediante el mecanismo de Obras por Impuestos y su contenido mínimo</t>
   </si>
   <si>
     <t>IDENTIFICÓ LA NORMA DE INTERÉS</t>
@@ -3186,7 +3249,7 @@
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3255,8 +3318,21 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3290,6 +3366,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3371,7 +3459,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3531,6 +3619,19 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4057,7 +4158,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:XFD1048576"/>
+  <dimension ref="A1:XFD1048573"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="3" customWidth="1"/>
@@ -12439,7 +12540,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="415" spans="1:6" ht="15">
+    <row r="415" spans="1:6">
       <c r="A415" s="3">
         <v>46203</v>
       </c>
@@ -12459,7 +12560,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="416" spans="1:6" ht="15">
+    <row r="416" spans="1:6">
       <c r="A416" s="3">
         <v>46203</v>
       </c>
@@ -12479,7 +12580,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="417" spans="1:6" ht="15">
+    <row r="417" spans="1:6">
       <c r="A417" s="3">
         <v>46203</v>
       </c>
@@ -12499,7 +12600,7 @@
         <v>838</v>
       </c>
     </row>
-    <row r="418" spans="1:6" ht="15">
+    <row r="418" spans="1:6">
       <c r="A418" s="3">
         <v>46203</v>
       </c>
@@ -12519,7 +12620,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="419" spans="1:6" ht="15">
+    <row r="419" spans="1:6">
       <c r="A419" s="3">
         <v>46203</v>
       </c>
@@ -12539,7 +12640,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="420" spans="1:6" ht="15">
+    <row r="420" spans="1:6">
       <c r="A420" s="3">
         <v>46204</v>
       </c>
@@ -12559,7 +12660,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="421" spans="1:6" ht="15">
+    <row r="421" spans="1:6">
       <c r="A421" s="3">
         <v>46204</v>
       </c>
@@ -12579,7 +12680,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="422" spans="1:6" ht="15">
+    <row r="422" spans="1:6">
       <c r="A422" s="3">
         <v>46204</v>
       </c>
@@ -12599,7 +12700,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="423" spans="1:6" ht="15">
+    <row r="423" spans="1:6">
       <c r="A423" s="3">
         <v>46204</v>
       </c>
@@ -12619,7 +12720,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="424" spans="1:6" ht="15">
+    <row r="424" spans="1:6">
       <c r="A424" s="3">
         <v>46204</v>
       </c>
@@ -12639,7 +12740,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="425" spans="1:6" ht="15">
+    <row r="425" spans="1:6">
       <c r="A425" s="3">
         <v>46205</v>
       </c>
@@ -12799,7 +12900,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="433" spans="1:6" ht="15">
+    <row r="433" spans="1:6">
       <c r="A433" s="3">
         <v>46207</v>
       </c>
@@ -12859,7 +12960,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="436" spans="1:6" ht="43.5">
+    <row r="436" spans="1:6" ht="29.1">
       <c r="A436" s="3">
         <v>46212</v>
       </c>
@@ -12939,7 +13040,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="440" spans="1:6" ht="29.25">
+    <row r="440" spans="1:6" ht="29.1">
       <c r="A440" s="3">
         <v>46217</v>
       </c>
@@ -12979,7 +13080,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="442" spans="1:6" ht="29.25">
+    <row r="442" spans="1:6" ht="29.1">
       <c r="A442" s="3">
         <v>46219</v>
       </c>
@@ -12999,7 +13100,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="443" spans="1:6" ht="29.25">
+    <row r="443" spans="1:6" ht="29.1">
       <c r="A443" s="3">
         <v>46219</v>
       </c>
@@ -13019,7 +13120,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="444" spans="1:6" ht="43.5">
+    <row r="444" spans="1:6" ht="29.1">
       <c r="A444" s="3">
         <v>46220</v>
       </c>
@@ -13039,7 +13140,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="445" spans="1:6" ht="57.75">
+    <row r="445" spans="1:6" ht="57.95">
       <c r="A445" s="3">
         <v>46223</v>
       </c>
@@ -13079,7 +13180,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="447" spans="1:6" ht="29.25">
+    <row r="447" spans="1:6" ht="29.1">
       <c r="A447" s="3">
         <v>46225</v>
       </c>
@@ -13099,7 +13200,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="448" spans="1:6" ht="29.25">
+    <row r="448" spans="1:6" ht="29.1">
       <c r="A448" s="3">
         <v>46226</v>
       </c>
@@ -13119,7 +13220,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="449" spans="1:6" ht="29.25">
+    <row r="449" spans="1:6" ht="29.1">
       <c r="A449" s="3">
         <v>46226</v>
       </c>
@@ -13139,7 +13240,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="450" spans="1:6" ht="57.75">
+    <row r="450" spans="1:6" ht="57.95">
       <c r="A450" s="3">
         <v>46226</v>
       </c>
@@ -13159,7 +13260,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="451" spans="1:6" ht="72.75">
+    <row r="451" spans="1:6" ht="57.95">
       <c r="A451" s="3">
         <v>46226</v>
       </c>
@@ -13179,7 +13280,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="452" spans="1:6" ht="29.25">
+    <row r="452" spans="1:6" ht="29.1">
       <c r="A452" s="3">
         <v>46227</v>
       </c>
@@ -13199,7 +13300,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="453" spans="1:6" ht="29.25">
+    <row r="453" spans="1:6" ht="29.1">
       <c r="A453" s="3">
         <v>46227</v>
       </c>
@@ -13219,7 +13320,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="454" spans="1:6" ht="43.5">
+    <row r="454" spans="1:6" ht="29.1">
       <c r="A454" s="3">
         <v>46228</v>
       </c>
@@ -13419,7 +13520,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="464" spans="1:6" ht="57.75">
+    <row r="464" spans="1:6" ht="57.95">
       <c r="A464" s="3">
         <v>46247</v>
       </c>
@@ -13439,7 +13540,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="465" spans="1:6" ht="87">
+    <row r="465" spans="1:6" ht="72.599999999999994">
       <c r="A465" s="3">
         <v>46247</v>
       </c>
@@ -13479,7 +13580,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="467" spans="1:6" s="58" customFormat="1" ht="15">
+    <row r="467" spans="1:6" s="58" customFormat="1">
       <c r="A467" s="61">
         <v>46249</v>
       </c>
@@ -13499,7 +13600,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="468" spans="1:6" ht="115.5">
+    <row r="468" spans="1:6" ht="87">
       <c r="A468" s="51">
         <v>46251</v>
       </c>
@@ -13579,7 +13680,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="472" spans="1:6" s="58" customFormat="1" ht="15">
+    <row r="472" spans="1:6" s="58" customFormat="1">
       <c r="A472" s="61">
         <v>46254</v>
       </c>
@@ -13779,23 +13880,23 @@
         <v>978</v>
       </c>
     </row>
-    <row r="482" spans="1:6" ht="29.25">
-      <c r="A482" s="3">
+    <row r="482" spans="1:6" ht="29.1">
+      <c r="A482" s="65">
         <v>46261</v>
       </c>
-      <c r="B482" t="s">
+      <c r="B482" s="66" t="s">
         <v>950</v>
       </c>
-      <c r="C482" t="s">
+      <c r="C482" s="66" t="s">
         <v>979</v>
       </c>
-      <c r="D482" t="s">
-        <v>29</v>
-      </c>
-      <c r="E482" t="s">
-        <v>30</v>
-      </c>
-      <c r="F482" s="45" t="s">
+      <c r="D482" s="66" t="s">
+        <v>29</v>
+      </c>
+      <c r="E482" s="66" t="s">
+        <v>30</v>
+      </c>
+      <c r="F482" s="67" t="s">
         <v>980</v>
       </c>
     </row>
@@ -13840,26 +13941,26 @@
       </c>
     </row>
     <row r="485" spans="1:6">
-      <c r="A485" s="3">
+      <c r="A485" s="62">
         <v>46262</v>
       </c>
-      <c r="B485" t="s">
+      <c r="B485" s="63" t="s">
         <v>984</v>
       </c>
-      <c r="C485" t="s">
+      <c r="C485" s="63" t="s">
         <v>985</v>
       </c>
-      <c r="D485" t="s">
-        <v>29</v>
-      </c>
-      <c r="E485" t="s">
+      <c r="D485" s="63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E485" s="63" t="s">
         <v>840</v>
       </c>
-      <c r="F485" s="4" t="s">
+      <c r="F485" s="64" t="s">
         <v>986</v>
       </c>
     </row>
-    <row r="486" spans="1:6" ht="101.25">
+    <row r="486" spans="1:6" ht="87">
       <c r="A486" s="54">
         <v>46262</v>
       </c>
@@ -13879,7 +13980,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="487" spans="1:6" ht="50.25">
+    <row r="487" spans="1:6" ht="51">
       <c r="A487" s="3">
         <v>46262</v>
       </c>
@@ -13899,7 +14000,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="488" spans="1:6" ht="24.75">
+    <row r="488" spans="1:6" ht="26.1">
       <c r="A488" s="3">
         <v>46262</v>
       </c>
@@ -13919,7 +14020,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="489" spans="1:6" ht="115.5">
+    <row r="489" spans="1:6" ht="101.45">
       <c r="A489" s="3">
         <v>46266</v>
       </c>
@@ -13939,7 +14040,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="490" spans="1:6" ht="29.25">
+    <row r="490" spans="1:6" ht="29.1">
       <c r="A490" s="3">
         <v>46266</v>
       </c>
@@ -13959,7 +14060,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="491" spans="1:6" ht="15">
+    <row r="491" spans="1:6">
       <c r="A491" s="3">
         <v>46266</v>
       </c>
@@ -13979,7 +14080,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="492" spans="1:6" ht="57.75">
+    <row r="492" spans="1:6" ht="43.5">
       <c r="A492" s="3">
         <v>46267</v>
       </c>
@@ -13999,16 +14100,172 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="493" spans="1:6">
+      <c r="A493" s="3">
+        <v>46269</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C493" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D493" t="s">
+        <v>29</v>
+      </c>
+      <c r="E493" t="s">
+        <v>30</v>
+      </c>
+      <c r="F493" s="4" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="494" spans="1:6">
+      <c r="A494" s="68">
+        <v>46262</v>
+      </c>
+      <c r="B494" s="69"/>
+      <c r="C494" s="68" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D494" s="69" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E494" s="69"/>
+      <c r="F494" s="69" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="495" spans="1:6" ht="101.25">
+      <c r="A495" s="3">
+        <v>46270</v>
+      </c>
+      <c r="B495" t="s">
+        <v>46</v>
+      </c>
+      <c r="C495" s="70" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D495" t="s">
+        <v>29</v>
+      </c>
+      <c r="E495" t="s">
+        <v>30</v>
+      </c>
+      <c r="F495" s="45" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="496" spans="1:6" ht="72.75">
+      <c r="A496" s="3">
+        <v>46270</v>
+      </c>
+      <c r="B496" t="s">
+        <v>46</v>
+      </c>
+      <c r="C496" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D496" t="s">
+        <v>29</v>
+      </c>
+      <c r="E496" t="s">
+        <v>30</v>
+      </c>
+      <c r="F496" s="45" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="497" spans="1:6">
+      <c r="A497" s="3">
+        <v>46275</v>
+      </c>
+      <c r="B497" t="s">
+        <v>49</v>
+      </c>
+      <c r="C497" t="s">
+        <v>1011</v>
+      </c>
+      <c r="D497" t="s">
+        <v>29</v>
+      </c>
+      <c r="E497" t="s">
+        <v>30</v>
+      </c>
+      <c r="F497" s="4" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="498" spans="1:6">
+      <c r="A498" s="3">
+        <v>46274</v>
+      </c>
+      <c r="B498" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C498" t="s">
+        <v>1014</v>
+      </c>
+      <c r="D498" t="s">
+        <v>29</v>
+      </c>
+      <c r="E498" t="s">
+        <v>30</v>
+      </c>
+      <c r="F498" s="4" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="499" spans="1:6">
+      <c r="A499" s="3">
+        <v>46274</v>
+      </c>
+      <c r="B499" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C499" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D499" t="s">
+        <v>29</v>
+      </c>
+      <c r="E499" t="s">
+        <v>30</v>
+      </c>
+      <c r="F499" s="4" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="500" spans="1:6">
+      <c r="A500" s="3">
+        <v>46274</v>
+      </c>
+      <c r="B500" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C500" t="s">
+        <v>1018</v>
+      </c>
+      <c r="D500" t="s">
+        <v>29</v>
+      </c>
+      <c r="E500" t="s">
+        <v>30</v>
+      </c>
+      <c r="F500" s="4" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="1048570" ht="12.75" customHeight="1"/>
+    <row r="1048571" ht="12.75" customHeight="1"/>
+    <row r="1048572" ht="12.75" customHeight="1"/>
     <row r="1048573" ht="12.75" customHeight="1"/>
-    <row r="1048574" ht="12.75" customHeight="1"/>
-    <row r="1048575" ht="12.75" customHeight="1"/>
-    <row r="1048576" ht="12.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:F492" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <conditionalFormatting sqref="C2">
     <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C28 C49:C414 C1 C420 C426:C466 C468:C471 C473:C486 C493:C1048576">
+  <conditionalFormatting sqref="C496:C1048576 C3:C28 C49:C414 C1 C420 C426:C466 C468:C471 C473:C486 F494 C493">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -14023,7 +14280,7 @@
   <sheetData>
     <row r="2" spans="2:8" ht="15" customHeight="1">
       <c r="D2" s="34" t="s">
-        <v>1001</v>
+        <v>1020</v>
       </c>
       <c r="E2" s="34"/>
     </row>
@@ -14032,10 +14289,10 @@
         <v>21</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>1002</v>
+        <v>1021</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>1003</v>
+        <v>1022</v>
       </c>
       <c r="E3" s="36" t="s">
         <v>24</v>
@@ -14044,44 +14301,44 @@
         <v>25</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>1004</v>
+        <v>1023</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>1005</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="362.45">
       <c r="B4" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>1007</v>
+        <v>1026</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>1009</v>
+        <v>1028</v>
       </c>
       <c r="H4" s="38" t="s">
-        <v>1010</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="304.5">
       <c r="B5" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>1011</v>
+        <v>1030</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>29</v>
@@ -14093,18 +14350,18 @@
         <v>31</v>
       </c>
       <c r="H5" s="40" t="s">
-        <v>1012</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="409.5">
       <c r="B6" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1013</v>
+        <v>1032</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>29</v>
@@ -14116,18 +14373,18 @@
         <v>34</v>
       </c>
       <c r="H6" s="41" t="s">
-        <v>1012</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="409.5">
       <c r="B7" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>1014</v>
+        <v>1033</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>29</v>
@@ -14139,15 +14396,15 @@
         <v>37</v>
       </c>
       <c r="H7" s="41" t="s">
-        <v>1012</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="409.5">
       <c r="B8" s="12" t="s">
-        <v>1015</v>
+        <v>1034</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1016</v>
+        <v>1035</v>
       </c>
       <c r="D8" s="42"/>
       <c r="E8" s="12" t="s">
@@ -14163,10 +14420,10 @@
     </row>
     <row r="9" spans="2:8" ht="409.5">
       <c r="B9" s="12" t="s">
-        <v>1015</v>
+        <v>1034</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1017</v>
+        <v>1036</v>
       </c>
       <c r="D9" s="42"/>
       <c r="E9" s="12" t="s">
@@ -14182,13 +14439,13 @@
     </row>
     <row r="10" spans="2:8" ht="409.5">
       <c r="B10" s="12" t="s">
-        <v>1018</v>
+        <v>1037</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1019</v>
+        <v>1038</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>29</v>
@@ -14203,55 +14460,55 @@
     </row>
     <row r="11" spans="2:8" ht="275.45">
       <c r="B11" s="12" t="s">
-        <v>1018</v>
+        <v>1037</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1020</v>
+        <v>1039</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="F11" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>1021</v>
+        <v>1040</v>
       </c>
       <c r="H11" s="42"/>
     </row>
     <row r="12" spans="2:8" ht="188.45">
       <c r="B12" s="12" t="s">
-        <v>1018</v>
+        <v>1037</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1022</v>
+        <v>1041</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="40" t="s">
-        <v>1023</v>
+        <v>1042</v>
       </c>
       <c r="H12" s="42"/>
     </row>
     <row r="13" spans="2:8" ht="409.5">
       <c r="B13" s="12" t="s">
-        <v>1024</v>
+        <v>1043</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>1025</v>
+        <v>1044</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E13" s="12" t="s">
         <v>29</v>
@@ -14260,7 +14517,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>1026</v>
+        <v>1045</v>
       </c>
       <c r="H13" s="42"/>
     </row>
@@ -14278,36 +14535,36 @@
   <sheetData>
     <row r="2" spans="2:8" ht="362.45">
       <c r="B2" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>1007</v>
+        <v>1026</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>1009</v>
+        <v>1028</v>
       </c>
       <c r="H2" s="38" t="s">
-        <v>1010</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="304.5">
       <c r="B3" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>1011</v>
+        <v>1030</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E3" s="12" t="s">
         <v>29</v>
@@ -14319,18 +14576,18 @@
         <v>31</v>
       </c>
       <c r="H3" s="40" t="s">
-        <v>1012</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="409.5">
       <c r="B4" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1013</v>
+        <v>1032</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>29</v>
@@ -14342,18 +14599,18 @@
         <v>34</v>
       </c>
       <c r="H4" s="41" t="s">
-        <v>1012</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="409.5">
       <c r="B5" s="12" t="s">
-        <v>1006</v>
+        <v>1025</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>1014</v>
+        <v>1033</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>29</v>
@@ -14365,15 +14622,15 @@
         <v>37</v>
       </c>
       <c r="H5" s="41" t="s">
-        <v>1012</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="409.5">
       <c r="B6" s="12" t="s">
-        <v>1015</v>
+        <v>1034</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1016</v>
+        <v>1035</v>
       </c>
       <c r="D6" s="42"/>
       <c r="E6" s="12" t="s">
@@ -14389,10 +14646,10 @@
     </row>
     <row r="7" spans="2:8" ht="409.5">
       <c r="B7" s="12" t="s">
-        <v>1015</v>
+        <v>1034</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1017</v>
+        <v>1036</v>
       </c>
       <c r="D7" s="42"/>
       <c r="E7" s="12" t="s">
@@ -14408,13 +14665,13 @@
     </row>
     <row r="8" spans="2:8" ht="409.5">
       <c r="B8" s="12" t="s">
-        <v>1018</v>
+        <v>1037</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1019</v>
+        <v>1038</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>29</v>
@@ -14429,55 +14686,55 @@
     </row>
     <row r="9" spans="2:8" ht="275.45">
       <c r="B9" s="12" t="s">
-        <v>1018</v>
+        <v>1037</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1020</v>
+        <v>1039</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="F9" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G9" s="40" t="s">
-        <v>1021</v>
+        <v>1040</v>
       </c>
       <c r="H9" s="42"/>
     </row>
     <row r="10" spans="2:8" ht="188.45">
       <c r="B10" s="12" t="s">
-        <v>1018</v>
+        <v>1037</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1022</v>
+        <v>1041</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>30</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>1023</v>
+        <v>1042</v>
       </c>
       <c r="H10" s="42"/>
     </row>
     <row r="11" spans="2:8" ht="409.5">
       <c r="B11" s="12" t="s">
-        <v>1024</v>
+        <v>1043</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1025</v>
+        <v>1044</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>1008</v>
+        <v>1027</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>29</v>
@@ -14486,7 +14743,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>1026</v>
+        <v>1045</v>
       </c>
       <c r="H11" s="42"/>
     </row>

</xml_diff>